<commit_message>
major cahnges in every retail booking screen and excel for discount field
</commit_message>
<xml_diff>
--- a/public/file/Trax Book Retail Shipment Template.xlsx
+++ b/public/file/Trax Book Retail Shipment Template.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26501"/>
+  <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\sonic\public\file\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9084FCFB-A219-4F4F-A475-0E31AE8ECD06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -24,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
   <si>
     <t>Consignee Name</t>
   </si>
@@ -111,12 +112,18 @@
   </si>
   <si>
     <t>Packaging Charges</t>
+  </si>
+  <si>
+    <t>Admin Discount Type</t>
+  </si>
+  <si>
+    <t>Admin Discount</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -471,8 +478,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AC1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:AE1"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.77734375" style="1" bestFit="1" customWidth="1"/>
@@ -501,9 +508,12 @@
     <col min="26" max="26" width="12.109375" style="1" bestFit="1" customWidth="1"/>
     <col min="27" max="27" width="14.77734375" style="1" bestFit="1" customWidth="1"/>
     <col min="28" max="28" width="10.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="14.5546875" customWidth="1"/>
+    <col min="30" max="30" width="13.77734375" customWidth="1"/>
+    <col min="31" max="31" width="17.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
@@ -590,6 +600,12 @@
       </c>
       <c r="AC1" s="1" t="s">
         <v>25</v>
+      </c>
+      <c r="AD1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="AE1" s="1" t="s">
+        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>